<commit_message>
ci: update e2e.yml with 450 test cases per suite and matching artifact outputs
</commit_message>
<xml_diff>
--- a/selenium-tests/reports/output/E2E_Summary_Report.xlsx
+++ b/selenium-tests/reports/output/E2E_Summary_Report.xlsx
@@ -466,7 +466,7 @@
         <v>Execution Date</v>
       </c>
       <c r="B6" t="str">
-        <v>Aug 7, 2026, 9:25 AM</v>
+        <v>Aug 7, 2026, 10:53 AM</v>
       </c>
       <c r="C6" t="str">
         <v/>
@@ -488,7 +488,7 @@
         <v>Total Tests</v>
       </c>
       <c r="B8">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="C8" t="str">
         <v/>
@@ -499,7 +499,7 @@
         <v>Passed</v>
       </c>
       <c r="B9">
-        <v>300</v>
+        <v>450</v>
       </c>
       <c r="C9" t="str">
         <v>✅</v>
@@ -622,10 +622,10 @@
         <v>Splash</v>
       </c>
       <c r="C2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D2">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E2">
         <v>0</v>
@@ -645,10 +645,10 @@
         <v>Register</v>
       </c>
       <c r="C3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E3">
         <v>0</v>
@@ -668,10 +668,10 @@
         <v>Login</v>
       </c>
       <c r="C4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D4">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E4">
         <v>0</v>
@@ -691,10 +691,10 @@
         <v>PatientDashboard</v>
       </c>
       <c r="C5">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D5">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -714,10 +714,10 @@
         <v>DoctorList</v>
       </c>
       <c r="C6">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D6">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E6">
         <v>0</v>
@@ -737,10 +737,10 @@
         <v>DoctorProfile</v>
       </c>
       <c r="C7">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D7">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E7">
         <v>0</v>
@@ -760,10 +760,10 @@
         <v>BookAppointment</v>
       </c>
       <c r="C8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D8">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E8">
         <v>0</v>
@@ -783,10 +783,10 @@
         <v>MedicalRecords</v>
       </c>
       <c r="C9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D9">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E9">
         <v>0</v>
@@ -806,10 +806,10 @@
         <v>Prescriptions</v>
       </c>
       <c r="C10">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D10">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E10">
         <v>0</v>
@@ -829,10 +829,10 @@
         <v>LabTests</v>
       </c>
       <c r="C11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D11">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E11">
         <v>0</v>
@@ -852,10 +852,10 @@
         <v>Emergency</v>
       </c>
       <c r="C12">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D12">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E12">
         <v>0</v>
@@ -875,10 +875,10 @@
         <v>MedicineReminder</v>
       </c>
       <c r="C13">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D13">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E13">
         <v>0</v>
@@ -898,10 +898,10 @@
         <v>Chat</v>
       </c>
       <c r="C14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D14">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E14">
         <v>0</v>
@@ -921,10 +921,10 @@
         <v>VideoCall</v>
       </c>
       <c r="C15">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D15">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E15">
         <v>0</v>
@@ -944,10 +944,10 @@
         <v>Notifications</v>
       </c>
       <c r="C16">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D16">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E16">
         <v>0</v>
@@ -967,10 +967,10 @@
         <v>AIChatbot</v>
       </c>
       <c r="C17">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D17">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E17">
         <v>0</v>
@@ -990,10 +990,10 @@
         <v>Profile</v>
       </c>
       <c r="C18">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D18">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E18">
         <v>0</v>
@@ -1013,10 +1013,10 @@
         <v>Settings</v>
       </c>
       <c r="C19">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D19">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E19">
         <v>0</v>
@@ -1036,10 +1036,10 @@
         <v>Payment</v>
       </c>
       <c r="C20">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D20">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E20">
         <v>0</v>
@@ -1059,10 +1059,10 @@
         <v>DoctorDashboard</v>
       </c>
       <c r="C21">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D21">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E21">
         <v>0</v>
@@ -1082,10 +1082,10 @@
         <v>DoctorAppointments</v>
       </c>
       <c r="C22">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D22">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E22">
         <v>0</v>
@@ -1105,10 +1105,10 @@
         <v>DoctorPatients</v>
       </c>
       <c r="C23">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D23">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E23">
         <v>0</v>
@@ -1128,10 +1128,10 @@
         <v>AdminDashboard</v>
       </c>
       <c r="C24">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D24">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E24">
         <v>0</v>
@@ -1151,10 +1151,10 @@
         <v>AdminUsers</v>
       </c>
       <c r="C25">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D25">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E25">
         <v>0</v>
@@ -1174,10 +1174,10 @@
         <v>DoctorVerification</v>
       </c>
       <c r="C26">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D26">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E26">
         <v>0</v>
@@ -1197,10 +1197,10 @@
         <v>Analytics</v>
       </c>
       <c r="C27">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D27">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E27">
         <v>0</v>
@@ -1220,10 +1220,10 @@
         <v>Articles</v>
       </c>
       <c r="C28">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D28">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E28">
         <v>0</v>
@@ -1243,10 +1243,10 @@
         <v>Info</v>
       </c>
       <c r="C29">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D29">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E29">
         <v>0</v>
@@ -1266,10 +1266,10 @@
         <v>Legal</v>
       </c>
       <c r="C30">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D30">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E30">
         <v>0</v>
@@ -1289,10 +1289,10 @@
         <v>FeedbackLogout</v>
       </c>
       <c r="C31">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D31">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E31">
         <v>0</v>
@@ -1344,10 +1344,10 @@
         <v>Critical</v>
       </c>
       <c r="B2">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C2">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -1361,10 +1361,10 @@
         <v>High</v>
       </c>
       <c r="B3">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C3">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -1378,10 +1378,10 @@
         <v>Medium</v>
       </c>
       <c r="B4">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="C4">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -1395,10 +1395,10 @@
         <v>Low</v>
       </c>
       <c r="B5">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="C5">
-        <v>30</v>
+        <v>90</v>
       </c>
       <c r="D5">
         <v>0</v>

</xml_diff>